<commit_message>
data updated on 2026-02-03 13:00:55.173256
</commit_message>
<xml_diff>
--- a/update_log.xlsx
+++ b/update_log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -626,6 +626,13 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:00:55</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data updated on 2026-02-09 11:53:44.300421
</commit_message>
<xml_diff>
--- a/update_log.xlsx
+++ b/update_log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -633,6 +633,13 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-02-09 11:53:44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revert "data updated on 2026-02-03 13:00:55.173256"
This reverts commit b59ec7aa7b64b63816a5756f9450672e5285c033.

# Conflicts:
#	update_log.xlsx
</commit_message>
<xml_diff>
--- a/update_log.xlsx
+++ b/update_log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -626,20 +626,6 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-02-03 13:00:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-02-09 11:53:44</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ALL FILES REVERT TO FEB 2 2026
</commit_message>
<xml_diff>
--- a/update_log.xlsx
+++ b/update_log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -626,6 +626,13 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:00:55</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated new models to test
</commit_message>
<xml_diff>
--- a/update_log.xlsx
+++ b/update_log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -633,6 +633,13 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:18:43</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>